<commit_message>
Allinea template di importazione a Odoo 20.0
- Conti bancari: account_number/holder_name/bank_name/bank_bic (res.bank
  non esiste più in 20): file istituti rimosso, unico 02_Conti_Bancari
- Dipendenti: employee_type_id (hr.employee.type), sex male/female,
  rimosso ssnid
- Manuale: riferimento 20.0 e tabella differenze 18/19/20

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013waGJG7pYcG8W9mHUJy7ny
</commit_message>
<xml_diff>
--- a/import_templates/03_Dipendenti.xlsx
+++ b/import_templates/03_Dipendenti.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dati" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valori" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +38,9 @@
     <font>
       <b val="1"/>
       <color rgb="00C0392B"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -93,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +119,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -305,8 +310,8 @@
       <text>
         <t>Tipo dipendente
 [Consigliato]
-Formato: employee
-Default: employee.</t>
+Formato: hr.contract_type_employee
+Odoo 20: anagrafica hr.employee.type. Vedi foglio Valori.</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
@@ -322,7 +327,7 @@
         <t>Data validità dati
 [Facoltativo]
 Formato: 2024-01-15
-Odoo 19: data di efficacia della "versione" del dipendente. Vuoto = oggi.</t>
+Odoo 20: data di efficacia della "versione" del dipendente. Vuoto = oggi.</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
@@ -335,21 +340,13 @@
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>N. previdenziale
+        <t>Sesso (legale)
 [Facoltativo]
-Formato: 
-Matricola INPS / altro, se usato.</t>
+Formato: male / female
+Sesso legale anagrafico (Odoo 20 ammette solo male/female).</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>Sesso
-[Facoltativo]
-Formato: male / female / other
-In Odoo 18 il campo si chiama gender.</t>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Data di nascita
 [Facoltativo]
@@ -357,7 +354,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Luogo di nascita
 [Facoltativo]
@@ -365,7 +362,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Paese di nascita
 [Facoltativo]
@@ -373,7 +370,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Nazionalità
 [Facoltativo]
@@ -381,7 +378,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Indirizzo privato
 [Facoltativo]
@@ -389,7 +386,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">CAP privato
 [Facoltativo]
@@ -397,7 +394,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Città privata
 [Facoltativo]
@@ -405,7 +402,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Provincia privata
 [Facoltativo]
@@ -413,7 +410,7 @@
 Usare base.state_it_ + sigla provincia minuscola: base.state_it_mi (Milano), base.state_it_rm (Roma), base.state_it_to (Torino)...</t>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Paese privato
 [Facoltativo]
@@ -421,7 +418,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Email privata
 [Facoltativo]
@@ -429,7 +426,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Telefono privato
 [Facoltativo]
@@ -437,7 +434,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
+    <comment ref="AD1" authorId="0" shapeId="0">
       <text>
         <t>Stato civile
 [Facoltativo]
@@ -445,7 +442,7 @@
 Default single.</t>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
+    <comment ref="AE1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Figli a carico
 [Facoltativo]
@@ -453,7 +450,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
+    <comment ref="AF1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Contatto emergenza
 [Facoltativo]
@@ -461,7 +458,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Tel. emergenza
 [Facoltativo]
@@ -469,7 +466,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AI1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Etichette
 [Facoltativo]
@@ -477,7 +474,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0">
+    <comment ref="AI1" authorId="0" shapeId="0">
       <text>
         <t>Badge ID
 [Facoltativo]
@@ -778,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ500"/>
+  <dimension ref="A1:AI500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -794,29 +791,28 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="21" customWidth="1" min="22" max="22"/>
-    <col width="15" customWidth="1" min="23" max="23"/>
-    <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="21" customWidth="1" min="27" max="27"/>
-    <col width="23" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
-    <col width="15" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="10" customWidth="1" min="32" max="32"/>
-    <col width="19" customWidth="1" min="33" max="33"/>
-    <col width="17" customWidth="1" min="34" max="34"/>
-    <col width="16" customWidth="1" min="35" max="35"/>
-    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="21" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="15" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="19" customWidth="1" min="32" max="32"/>
+    <col width="17" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="10" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -887,7 +883,7 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>employee_type</t>
+          <t>employee_type_id/id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -907,95 +903,90 @@
       </c>
       <c r="R1" s="3" t="inlineStr">
         <is>
-          <t>ssnid</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="S1" s="3" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>birthday</t>
         </is>
       </c>
       <c r="T1" s="3" t="inlineStr">
         <is>
-          <t>birthday</t>
+          <t>place_of_birth</t>
         </is>
       </c>
       <c r="U1" s="3" t="inlineStr">
         <is>
-          <t>place_of_birth</t>
+          <t>country_of_birth/id</t>
         </is>
       </c>
       <c r="V1" s="3" t="inlineStr">
         <is>
-          <t>country_of_birth/id</t>
+          <t>country_id/id</t>
         </is>
       </c>
       <c r="W1" s="3" t="inlineStr">
         <is>
-          <t>country_id/id</t>
+          <t>private_street</t>
         </is>
       </c>
       <c r="X1" s="3" t="inlineStr">
         <is>
-          <t>private_street</t>
+          <t>private_zip</t>
         </is>
       </c>
       <c r="Y1" s="3" t="inlineStr">
         <is>
-          <t>private_zip</t>
+          <t>private_city</t>
         </is>
       </c>
       <c r="Z1" s="3" t="inlineStr">
         <is>
-          <t>private_city</t>
+          <t>private_state_id/id</t>
         </is>
       </c>
       <c r="AA1" s="3" t="inlineStr">
         <is>
-          <t>private_state_id/id</t>
+          <t>private_country_id/id</t>
         </is>
       </c>
       <c r="AB1" s="3" t="inlineStr">
         <is>
-          <t>private_country_id/id</t>
+          <t>private_email</t>
         </is>
       </c>
       <c r="AC1" s="3" t="inlineStr">
         <is>
-          <t>private_email</t>
+          <t>private_phone</t>
         </is>
       </c>
       <c r="AD1" s="3" t="inlineStr">
         <is>
-          <t>private_phone</t>
+          <t>marital</t>
         </is>
       </c>
       <c r="AE1" s="3" t="inlineStr">
         <is>
-          <t>marital</t>
+          <t>children</t>
         </is>
       </c>
       <c r="AF1" s="3" t="inlineStr">
         <is>
-          <t>children</t>
+          <t>emergency_contact</t>
         </is>
       </c>
       <c r="AG1" s="3" t="inlineStr">
         <is>
-          <t>emergency_contact</t>
+          <t>emergency_phone</t>
         </is>
       </c>
       <c r="AH1" s="3" t="inlineStr">
         <is>
-          <t>emergency_phone</t>
+          <t>category_ids</t>
         </is>
       </c>
       <c r="AI1" s="3" t="inlineStr">
-        <is>
-          <t>category_ids</t>
-        </is>
-      </c>
-      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>barcode</t>
         </is>
@@ -1041,7 +1032,7 @@
       <c r="M2" s="4" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>employee</t>
+          <t>hr.contract_type_employee</t>
         </is>
       </c>
       <c r="O2" s="4" t="inlineStr">
@@ -1055,20 +1046,24 @@
           <t>BNCLRA85C41F205X</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr"/>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>female</t>
+          <t>1985-03-01</t>
         </is>
       </c>
       <c r="T2" s="4" t="inlineStr">
         <is>
-          <t>1985-03-01</t>
+          <t>Milano</t>
         </is>
       </c>
       <c r="U2" s="4" t="inlineStr">
         <is>
-          <t>Milano</t>
+          <t>base.it</t>
         </is>
       </c>
       <c r="V2" s="4" t="inlineStr">
@@ -1076,34 +1071,29 @@
           <t>base.it</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr"/>
+      <c r="X2" s="5" t="inlineStr"/>
+      <c r="Y2" s="4" t="inlineStr"/>
+      <c r="Z2" s="4" t="inlineStr"/>
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>base.it</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr"/>
-      <c r="Y2" s="5" t="inlineStr"/>
-      <c r="Z2" s="4" t="inlineStr"/>
-      <c r="AA2" s="4" t="inlineStr"/>
-      <c r="AB2" s="4" t="inlineStr">
-        <is>
-          <t>base.it</t>
-        </is>
-      </c>
+      <c r="AB2" s="4" t="inlineStr"/>
       <c r="AC2" s="4" t="inlineStr"/>
-      <c r="AD2" s="4" t="inlineStr"/>
-      <c r="AE2" s="4" t="inlineStr">
+      <c r="AD2" s="4" t="inlineStr">
         <is>
           <t>married</t>
         </is>
       </c>
-      <c r="AF2" s="4" t="n">
+      <c r="AE2" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="AF2" s="4" t="inlineStr"/>
       <c r="AG2" s="4" t="inlineStr"/>
       <c r="AH2" s="4" t="inlineStr"/>
-      <c r="AI2" s="4" t="inlineStr"/>
-      <c r="AJ2" s="5" t="inlineStr"/>
+      <c r="AI2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1149,7 +1139,7 @@
       <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>employee</t>
+          <t>hr.contract_type_employee</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -1163,20 +1153,24 @@
           <t>VRDPLA90A01L219Z</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr"/>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
       <c r="S3" s="4" t="inlineStr">
         <is>
-          <t>male</t>
+          <t>1990-01-01</t>
         </is>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>1990-01-01</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>base.it</t>
         </is>
       </c>
       <c r="V3" s="4" t="inlineStr">
@@ -1184,1535 +1178,1530 @@
           <t>base.it</t>
         </is>
       </c>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="W3" s="4" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="4" t="inlineStr"/>
+      <c r="Z3" s="4" t="inlineStr"/>
+      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>base.it</t>
         </is>
       </c>
-      <c r="X3" s="4" t="inlineStr"/>
-      <c r="Y3" s="5" t="inlineStr"/>
-      <c r="Z3" s="4" t="inlineStr"/>
-      <c r="AA3" s="4" t="inlineStr"/>
-      <c r="AB3" s="4" t="inlineStr">
-        <is>
-          <t>base.it</t>
-        </is>
-      </c>
+      <c r="AB3" s="4" t="inlineStr"/>
       <c r="AC3" s="4" t="inlineStr"/>
-      <c r="AD3" s="4" t="inlineStr"/>
-      <c r="AE3" s="4" t="inlineStr">
+      <c r="AD3" s="4" t="inlineStr">
         <is>
           <t>single</t>
         </is>
       </c>
-      <c r="AF3" s="4" t="n">
+      <c r="AE3" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AF3" s="4" t="inlineStr"/>
       <c r="AG3" s="4" t="inlineStr"/>
       <c r="AH3" s="4" t="inlineStr"/>
-      <c r="AI3" s="4" t="inlineStr"/>
-      <c r="AJ3" s="5" t="inlineStr"/>
+      <c r="AI3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="Y4" s="6" t="n"/>
+      <c r="X4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="Y5" s="6" t="n"/>
+      <c r="X5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="Y6" s="6" t="n"/>
+      <c r="X6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="Y7" s="6" t="n"/>
+      <c r="X7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="Y8" s="6" t="n"/>
+      <c r="X8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="Y9" s="6" t="n"/>
+      <c r="X9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="Y10" s="6" t="n"/>
+      <c r="X10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="Y11" s="6" t="n"/>
+      <c r="X11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="Y12" s="6" t="n"/>
+      <c r="X12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="Y13" s="6" t="n"/>
+      <c r="X13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="Y14" s="6" t="n"/>
+      <c r="X14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="Y15" s="6" t="n"/>
+      <c r="X15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="Y16" s="6" t="n"/>
+      <c r="X16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="Y17" s="6" t="n"/>
+      <c r="X17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="Y18" s="6" t="n"/>
+      <c r="X18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="Y19" s="6" t="n"/>
+      <c r="X19" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="Y20" s="6" t="n"/>
+      <c r="X20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="Y21" s="6" t="n"/>
+      <c r="X21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="Y22" s="6" t="n"/>
+      <c r="X22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="Y23" s="6" t="n"/>
+      <c r="X23" s="6" t="n"/>
     </row>
     <row r="24">
-      <c r="Y24" s="6" t="n"/>
+      <c r="X24" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="Y25" s="6" t="n"/>
+      <c r="X25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="Y26" s="6" t="n"/>
+      <c r="X26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="Y27" s="6" t="n"/>
+      <c r="X27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="Y28" s="6" t="n"/>
+      <c r="X28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="Y29" s="6" t="n"/>
+      <c r="X29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="Y30" s="6" t="n"/>
+      <c r="X30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="Y31" s="6" t="n"/>
+      <c r="X31" s="6" t="n"/>
     </row>
     <row r="32">
-      <c r="Y32" s="6" t="n"/>
+      <c r="X32" s="6" t="n"/>
     </row>
     <row r="33">
-      <c r="Y33" s="6" t="n"/>
+      <c r="X33" s="6" t="n"/>
     </row>
     <row r="34">
-      <c r="Y34" s="6" t="n"/>
+      <c r="X34" s="6" t="n"/>
     </row>
     <row r="35">
-      <c r="Y35" s="6" t="n"/>
+      <c r="X35" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="Y36" s="6" t="n"/>
+      <c r="X36" s="6" t="n"/>
     </row>
     <row r="37">
-      <c r="Y37" s="6" t="n"/>
+      <c r="X37" s="6" t="n"/>
     </row>
     <row r="38">
-      <c r="Y38" s="6" t="n"/>
+      <c r="X38" s="6" t="n"/>
     </row>
     <row r="39">
-      <c r="Y39" s="6" t="n"/>
+      <c r="X39" s="6" t="n"/>
     </row>
     <row r="40">
-      <c r="Y40" s="6" t="n"/>
+      <c r="X40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="Y41" s="6" t="n"/>
+      <c r="X41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="Y42" s="6" t="n"/>
+      <c r="X42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="Y43" s="6" t="n"/>
+      <c r="X43" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="Y44" s="6" t="n"/>
+      <c r="X44" s="6" t="n"/>
     </row>
     <row r="45">
-      <c r="Y45" s="6" t="n"/>
+      <c r="X45" s="6" t="n"/>
     </row>
     <row r="46">
-      <c r="Y46" s="6" t="n"/>
+      <c r="X46" s="6" t="n"/>
     </row>
     <row r="47">
-      <c r="Y47" s="6" t="n"/>
+      <c r="X47" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="Y48" s="6" t="n"/>
+      <c r="X48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="Y49" s="6" t="n"/>
+      <c r="X49" s="6" t="n"/>
     </row>
     <row r="50">
-      <c r="Y50" s="6" t="n"/>
+      <c r="X50" s="6" t="n"/>
     </row>
     <row r="51">
-      <c r="Y51" s="6" t="n"/>
+      <c r="X51" s="6" t="n"/>
     </row>
     <row r="52">
-      <c r="Y52" s="6" t="n"/>
+      <c r="X52" s="6" t="n"/>
     </row>
     <row r="53">
-      <c r="Y53" s="6" t="n"/>
+      <c r="X53" s="6" t="n"/>
     </row>
     <row r="54">
-      <c r="Y54" s="6" t="n"/>
+      <c r="X54" s="6" t="n"/>
     </row>
     <row r="55">
-      <c r="Y55" s="6" t="n"/>
+      <c r="X55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="Y56" s="6" t="n"/>
+      <c r="X56" s="6" t="n"/>
     </row>
     <row r="57">
-      <c r="Y57" s="6" t="n"/>
+      <c r="X57" s="6" t="n"/>
     </row>
     <row r="58">
-      <c r="Y58" s="6" t="n"/>
+      <c r="X58" s="6" t="n"/>
     </row>
     <row r="59">
-      <c r="Y59" s="6" t="n"/>
+      <c r="X59" s="6" t="n"/>
     </row>
     <row r="60">
-      <c r="Y60" s="6" t="n"/>
+      <c r="X60" s="6" t="n"/>
     </row>
     <row r="61">
-      <c r="Y61" s="6" t="n"/>
+      <c r="X61" s="6" t="n"/>
     </row>
     <row r="62">
-      <c r="Y62" s="6" t="n"/>
+      <c r="X62" s="6" t="n"/>
     </row>
     <row r="63">
-      <c r="Y63" s="6" t="n"/>
+      <c r="X63" s="6" t="n"/>
     </row>
     <row r="64">
-      <c r="Y64" s="6" t="n"/>
+      <c r="X64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="Y65" s="6" t="n"/>
+      <c r="X65" s="6" t="n"/>
     </row>
     <row r="66">
-      <c r="Y66" s="6" t="n"/>
+      <c r="X66" s="6" t="n"/>
     </row>
     <row r="67">
-      <c r="Y67" s="6" t="n"/>
+      <c r="X67" s="6" t="n"/>
     </row>
     <row r="68">
-      <c r="Y68" s="6" t="n"/>
+      <c r="X68" s="6" t="n"/>
     </row>
     <row r="69">
-      <c r="Y69" s="6" t="n"/>
+      <c r="X69" s="6" t="n"/>
     </row>
     <row r="70">
-      <c r="Y70" s="6" t="n"/>
+      <c r="X70" s="6" t="n"/>
     </row>
     <row r="71">
-      <c r="Y71" s="6" t="n"/>
+      <c r="X71" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="Y72" s="6" t="n"/>
+      <c r="X72" s="6" t="n"/>
     </row>
     <row r="73">
-      <c r="Y73" s="6" t="n"/>
+      <c r="X73" s="6" t="n"/>
     </row>
     <row r="74">
-      <c r="Y74" s="6" t="n"/>
+      <c r="X74" s="6" t="n"/>
     </row>
     <row r="75">
-      <c r="Y75" s="6" t="n"/>
+      <c r="X75" s="6" t="n"/>
     </row>
     <row r="76">
-      <c r="Y76" s="6" t="n"/>
+      <c r="X76" s="6" t="n"/>
     </row>
     <row r="77">
-      <c r="Y77" s="6" t="n"/>
+      <c r="X77" s="6" t="n"/>
     </row>
     <row r="78">
-      <c r="Y78" s="6" t="n"/>
+      <c r="X78" s="6" t="n"/>
     </row>
     <row r="79">
-      <c r="Y79" s="6" t="n"/>
+      <c r="X79" s="6" t="n"/>
     </row>
     <row r="80">
-      <c r="Y80" s="6" t="n"/>
+      <c r="X80" s="6" t="n"/>
     </row>
     <row r="81">
-      <c r="Y81" s="6" t="n"/>
+      <c r="X81" s="6" t="n"/>
     </row>
     <row r="82">
-      <c r="Y82" s="6" t="n"/>
+      <c r="X82" s="6" t="n"/>
     </row>
     <row r="83">
-      <c r="Y83" s="6" t="n"/>
+      <c r="X83" s="6" t="n"/>
     </row>
     <row r="84">
-      <c r="Y84" s="6" t="n"/>
+      <c r="X84" s="6" t="n"/>
     </row>
     <row r="85">
-      <c r="Y85" s="6" t="n"/>
+      <c r="X85" s="6" t="n"/>
     </row>
     <row r="86">
-      <c r="Y86" s="6" t="n"/>
+      <c r="X86" s="6" t="n"/>
     </row>
     <row r="87">
-      <c r="Y87" s="6" t="n"/>
+      <c r="X87" s="6" t="n"/>
     </row>
     <row r="88">
-      <c r="Y88" s="6" t="n"/>
+      <c r="X88" s="6" t="n"/>
     </row>
     <row r="89">
-      <c r="Y89" s="6" t="n"/>
+      <c r="X89" s="6" t="n"/>
     </row>
     <row r="90">
-      <c r="Y90" s="6" t="n"/>
+      <c r="X90" s="6" t="n"/>
     </row>
     <row r="91">
-      <c r="Y91" s="6" t="n"/>
+      <c r="X91" s="6" t="n"/>
     </row>
     <row r="92">
-      <c r="Y92" s="6" t="n"/>
+      <c r="X92" s="6" t="n"/>
     </row>
     <row r="93">
-      <c r="Y93" s="6" t="n"/>
+      <c r="X93" s="6" t="n"/>
     </row>
     <row r="94">
-      <c r="Y94" s="6" t="n"/>
+      <c r="X94" s="6" t="n"/>
     </row>
     <row r="95">
-      <c r="Y95" s="6" t="n"/>
+      <c r="X95" s="6" t="n"/>
     </row>
     <row r="96">
-      <c r="Y96" s="6" t="n"/>
+      <c r="X96" s="6" t="n"/>
     </row>
     <row r="97">
-      <c r="Y97" s="6" t="n"/>
+      <c r="X97" s="6" t="n"/>
     </row>
     <row r="98">
-      <c r="Y98" s="6" t="n"/>
+      <c r="X98" s="6" t="n"/>
     </row>
     <row r="99">
-      <c r="Y99" s="6" t="n"/>
+      <c r="X99" s="6" t="n"/>
     </row>
     <row r="100">
-      <c r="Y100" s="6" t="n"/>
+      <c r="X100" s="6" t="n"/>
     </row>
     <row r="101">
-      <c r="Y101" s="6" t="n"/>
+      <c r="X101" s="6" t="n"/>
     </row>
     <row r="102">
-      <c r="Y102" s="6" t="n"/>
+      <c r="X102" s="6" t="n"/>
     </row>
     <row r="103">
-      <c r="Y103" s="6" t="n"/>
+      <c r="X103" s="6" t="n"/>
     </row>
     <row r="104">
-      <c r="Y104" s="6" t="n"/>
+      <c r="X104" s="6" t="n"/>
     </row>
     <row r="105">
-      <c r="Y105" s="6" t="n"/>
+      <c r="X105" s="6" t="n"/>
     </row>
     <row r="106">
-      <c r="Y106" s="6" t="n"/>
+      <c r="X106" s="6" t="n"/>
     </row>
     <row r="107">
-      <c r="Y107" s="6" t="n"/>
+      <c r="X107" s="6" t="n"/>
     </row>
     <row r="108">
-      <c r="Y108" s="6" t="n"/>
+      <c r="X108" s="6" t="n"/>
     </row>
     <row r="109">
-      <c r="Y109" s="6" t="n"/>
+      <c r="X109" s="6" t="n"/>
     </row>
     <row r="110">
-      <c r="Y110" s="6" t="n"/>
+      <c r="X110" s="6" t="n"/>
     </row>
     <row r="111">
-      <c r="Y111" s="6" t="n"/>
+      <c r="X111" s="6" t="n"/>
     </row>
     <row r="112">
-      <c r="Y112" s="6" t="n"/>
+      <c r="X112" s="6" t="n"/>
     </row>
     <row r="113">
-      <c r="Y113" s="6" t="n"/>
+      <c r="X113" s="6" t="n"/>
     </row>
     <row r="114">
-      <c r="Y114" s="6" t="n"/>
+      <c r="X114" s="6" t="n"/>
     </row>
     <row r="115">
-      <c r="Y115" s="6" t="n"/>
+      <c r="X115" s="6" t="n"/>
     </row>
     <row r="116">
-      <c r="Y116" s="6" t="n"/>
+      <c r="X116" s="6" t="n"/>
     </row>
     <row r="117">
-      <c r="Y117" s="6" t="n"/>
+      <c r="X117" s="6" t="n"/>
     </row>
     <row r="118">
-      <c r="Y118" s="6" t="n"/>
+      <c r="X118" s="6" t="n"/>
     </row>
     <row r="119">
-      <c r="Y119" s="6" t="n"/>
+      <c r="X119" s="6" t="n"/>
     </row>
     <row r="120">
-      <c r="Y120" s="6" t="n"/>
+      <c r="X120" s="6" t="n"/>
     </row>
     <row r="121">
-      <c r="Y121" s="6" t="n"/>
+      <c r="X121" s="6" t="n"/>
     </row>
     <row r="122">
-      <c r="Y122" s="6" t="n"/>
+      <c r="X122" s="6" t="n"/>
     </row>
     <row r="123">
-      <c r="Y123" s="6" t="n"/>
+      <c r="X123" s="6" t="n"/>
     </row>
     <row r="124">
-      <c r="Y124" s="6" t="n"/>
+      <c r="X124" s="6" t="n"/>
     </row>
     <row r="125">
-      <c r="Y125" s="6" t="n"/>
+      <c r="X125" s="6" t="n"/>
     </row>
     <row r="126">
-      <c r="Y126" s="6" t="n"/>
+      <c r="X126" s="6" t="n"/>
     </row>
     <row r="127">
-      <c r="Y127" s="6" t="n"/>
+      <c r="X127" s="6" t="n"/>
     </row>
     <row r="128">
-      <c r="Y128" s="6" t="n"/>
+      <c r="X128" s="6" t="n"/>
     </row>
     <row r="129">
-      <c r="Y129" s="6" t="n"/>
+      <c r="X129" s="6" t="n"/>
     </row>
     <row r="130">
-      <c r="Y130" s="6" t="n"/>
+      <c r="X130" s="6" t="n"/>
     </row>
     <row r="131">
-      <c r="Y131" s="6" t="n"/>
+      <c r="X131" s="6" t="n"/>
     </row>
     <row r="132">
-      <c r="Y132" s="6" t="n"/>
+      <c r="X132" s="6" t="n"/>
     </row>
     <row r="133">
-      <c r="Y133" s="6" t="n"/>
+      <c r="X133" s="6" t="n"/>
     </row>
     <row r="134">
-      <c r="Y134" s="6" t="n"/>
+      <c r="X134" s="6" t="n"/>
     </row>
     <row r="135">
-      <c r="Y135" s="6" t="n"/>
+      <c r="X135" s="6" t="n"/>
     </row>
     <row r="136">
-      <c r="Y136" s="6" t="n"/>
+      <c r="X136" s="6" t="n"/>
     </row>
     <row r="137">
-      <c r="Y137" s="6" t="n"/>
+      <c r="X137" s="6" t="n"/>
     </row>
     <row r="138">
-      <c r="Y138" s="6" t="n"/>
+      <c r="X138" s="6" t="n"/>
     </row>
     <row r="139">
-      <c r="Y139" s="6" t="n"/>
+      <c r="X139" s="6" t="n"/>
     </row>
     <row r="140">
-      <c r="Y140" s="6" t="n"/>
+      <c r="X140" s="6" t="n"/>
     </row>
     <row r="141">
-      <c r="Y141" s="6" t="n"/>
+      <c r="X141" s="6" t="n"/>
     </row>
     <row r="142">
-      <c r="Y142" s="6" t="n"/>
+      <c r="X142" s="6" t="n"/>
     </row>
     <row r="143">
-      <c r="Y143" s="6" t="n"/>
+      <c r="X143" s="6" t="n"/>
     </row>
     <row r="144">
-      <c r="Y144" s="6" t="n"/>
+      <c r="X144" s="6" t="n"/>
     </row>
     <row r="145">
-      <c r="Y145" s="6" t="n"/>
+      <c r="X145" s="6" t="n"/>
     </row>
     <row r="146">
-      <c r="Y146" s="6" t="n"/>
+      <c r="X146" s="6" t="n"/>
     </row>
     <row r="147">
-      <c r="Y147" s="6" t="n"/>
+      <c r="X147" s="6" t="n"/>
     </row>
     <row r="148">
-      <c r="Y148" s="6" t="n"/>
+      <c r="X148" s="6" t="n"/>
     </row>
     <row r="149">
-      <c r="Y149" s="6" t="n"/>
+      <c r="X149" s="6" t="n"/>
     </row>
     <row r="150">
-      <c r="Y150" s="6" t="n"/>
+      <c r="X150" s="6" t="n"/>
     </row>
     <row r="151">
-      <c r="Y151" s="6" t="n"/>
+      <c r="X151" s="6" t="n"/>
     </row>
     <row r="152">
-      <c r="Y152" s="6" t="n"/>
+      <c r="X152" s="6" t="n"/>
     </row>
     <row r="153">
-      <c r="Y153" s="6" t="n"/>
+      <c r="X153" s="6" t="n"/>
     </row>
     <row r="154">
-      <c r="Y154" s="6" t="n"/>
+      <c r="X154" s="6" t="n"/>
     </row>
     <row r="155">
-      <c r="Y155" s="6" t="n"/>
+      <c r="X155" s="6" t="n"/>
     </row>
     <row r="156">
-      <c r="Y156" s="6" t="n"/>
+      <c r="X156" s="6" t="n"/>
     </row>
     <row r="157">
-      <c r="Y157" s="6" t="n"/>
+      <c r="X157" s="6" t="n"/>
     </row>
     <row r="158">
-      <c r="Y158" s="6" t="n"/>
+      <c r="X158" s="6" t="n"/>
     </row>
     <row r="159">
-      <c r="Y159" s="6" t="n"/>
+      <c r="X159" s="6" t="n"/>
     </row>
     <row r="160">
-      <c r="Y160" s="6" t="n"/>
+      <c r="X160" s="6" t="n"/>
     </row>
     <row r="161">
-      <c r="Y161" s="6" t="n"/>
+      <c r="X161" s="6" t="n"/>
     </row>
     <row r="162">
-      <c r="Y162" s="6" t="n"/>
+      <c r="X162" s="6" t="n"/>
     </row>
     <row r="163">
-      <c r="Y163" s="6" t="n"/>
+      <c r="X163" s="6" t="n"/>
     </row>
     <row r="164">
-      <c r="Y164" s="6" t="n"/>
+      <c r="X164" s="6" t="n"/>
     </row>
     <row r="165">
-      <c r="Y165" s="6" t="n"/>
+      <c r="X165" s="6" t="n"/>
     </row>
     <row r="166">
-      <c r="Y166" s="6" t="n"/>
+      <c r="X166" s="6" t="n"/>
     </row>
     <row r="167">
-      <c r="Y167" s="6" t="n"/>
+      <c r="X167" s="6" t="n"/>
     </row>
     <row r="168">
-      <c r="Y168" s="6" t="n"/>
+      <c r="X168" s="6" t="n"/>
     </row>
     <row r="169">
-      <c r="Y169" s="6" t="n"/>
+      <c r="X169" s="6" t="n"/>
     </row>
     <row r="170">
-      <c r="Y170" s="6" t="n"/>
+      <c r="X170" s="6" t="n"/>
     </row>
     <row r="171">
-      <c r="Y171" s="6" t="n"/>
+      <c r="X171" s="6" t="n"/>
     </row>
     <row r="172">
-      <c r="Y172" s="6" t="n"/>
+      <c r="X172" s="6" t="n"/>
     </row>
     <row r="173">
-      <c r="Y173" s="6" t="n"/>
+      <c r="X173" s="6" t="n"/>
     </row>
     <row r="174">
-      <c r="Y174" s="6" t="n"/>
+      <c r="X174" s="6" t="n"/>
     </row>
     <row r="175">
-      <c r="Y175" s="6" t="n"/>
+      <c r="X175" s="6" t="n"/>
     </row>
     <row r="176">
-      <c r="Y176" s="6" t="n"/>
+      <c r="X176" s="6" t="n"/>
     </row>
     <row r="177">
-      <c r="Y177" s="6" t="n"/>
+      <c r="X177" s="6" t="n"/>
     </row>
     <row r="178">
-      <c r="Y178" s="6" t="n"/>
+      <c r="X178" s="6" t="n"/>
     </row>
     <row r="179">
-      <c r="Y179" s="6" t="n"/>
+      <c r="X179" s="6" t="n"/>
     </row>
     <row r="180">
-      <c r="Y180" s="6" t="n"/>
+      <c r="X180" s="6" t="n"/>
     </row>
     <row r="181">
-      <c r="Y181" s="6" t="n"/>
+      <c r="X181" s="6" t="n"/>
     </row>
     <row r="182">
-      <c r="Y182" s="6" t="n"/>
+      <c r="X182" s="6" t="n"/>
     </row>
     <row r="183">
-      <c r="Y183" s="6" t="n"/>
+      <c r="X183" s="6" t="n"/>
     </row>
     <row r="184">
-      <c r="Y184" s="6" t="n"/>
+      <c r="X184" s="6" t="n"/>
     </row>
     <row r="185">
-      <c r="Y185" s="6" t="n"/>
+      <c r="X185" s="6" t="n"/>
     </row>
     <row r="186">
-      <c r="Y186" s="6" t="n"/>
+      <c r="X186" s="6" t="n"/>
     </row>
     <row r="187">
-      <c r="Y187" s="6" t="n"/>
+      <c r="X187" s="6" t="n"/>
     </row>
     <row r="188">
-      <c r="Y188" s="6" t="n"/>
+      <c r="X188" s="6" t="n"/>
     </row>
     <row r="189">
-      <c r="Y189" s="6" t="n"/>
+      <c r="X189" s="6" t="n"/>
     </row>
     <row r="190">
-      <c r="Y190" s="6" t="n"/>
+      <c r="X190" s="6" t="n"/>
     </row>
     <row r="191">
-      <c r="Y191" s="6" t="n"/>
+      <c r="X191" s="6" t="n"/>
     </row>
     <row r="192">
-      <c r="Y192" s="6" t="n"/>
+      <c r="X192" s="6" t="n"/>
     </row>
     <row r="193">
-      <c r="Y193" s="6" t="n"/>
+      <c r="X193" s="6" t="n"/>
     </row>
     <row r="194">
-      <c r="Y194" s="6" t="n"/>
+      <c r="X194" s="6" t="n"/>
     </row>
     <row r="195">
-      <c r="Y195" s="6" t="n"/>
+      <c r="X195" s="6" t="n"/>
     </row>
     <row r="196">
-      <c r="Y196" s="6" t="n"/>
+      <c r="X196" s="6" t="n"/>
     </row>
     <row r="197">
-      <c r="Y197" s="6" t="n"/>
+      <c r="X197" s="6" t="n"/>
     </row>
     <row r="198">
-      <c r="Y198" s="6" t="n"/>
+      <c r="X198" s="6" t="n"/>
     </row>
     <row r="199">
-      <c r="Y199" s="6" t="n"/>
+      <c r="X199" s="6" t="n"/>
     </row>
     <row r="200">
-      <c r="Y200" s="6" t="n"/>
+      <c r="X200" s="6" t="n"/>
     </row>
     <row r="201">
-      <c r="Y201" s="6" t="n"/>
+      <c r="X201" s="6" t="n"/>
     </row>
     <row r="202">
-      <c r="Y202" s="6" t="n"/>
+      <c r="X202" s="6" t="n"/>
     </row>
     <row r="203">
-      <c r="Y203" s="6" t="n"/>
+      <c r="X203" s="6" t="n"/>
     </row>
     <row r="204">
-      <c r="Y204" s="6" t="n"/>
+      <c r="X204" s="6" t="n"/>
     </row>
     <row r="205">
-      <c r="Y205" s="6" t="n"/>
+      <c r="X205" s="6" t="n"/>
     </row>
     <row r="206">
-      <c r="Y206" s="6" t="n"/>
+      <c r="X206" s="6" t="n"/>
     </row>
     <row r="207">
-      <c r="Y207" s="6" t="n"/>
+      <c r="X207" s="6" t="n"/>
     </row>
     <row r="208">
-      <c r="Y208" s="6" t="n"/>
+      <c r="X208" s="6" t="n"/>
     </row>
     <row r="209">
-      <c r="Y209" s="6" t="n"/>
+      <c r="X209" s="6" t="n"/>
     </row>
     <row r="210">
-      <c r="Y210" s="6" t="n"/>
+      <c r="X210" s="6" t="n"/>
     </row>
     <row r="211">
-      <c r="Y211" s="6" t="n"/>
+      <c r="X211" s="6" t="n"/>
     </row>
     <row r="212">
-      <c r="Y212" s="6" t="n"/>
+      <c r="X212" s="6" t="n"/>
     </row>
     <row r="213">
-      <c r="Y213" s="6" t="n"/>
+      <c r="X213" s="6" t="n"/>
     </row>
     <row r="214">
-      <c r="Y214" s="6" t="n"/>
+      <c r="X214" s="6" t="n"/>
     </row>
     <row r="215">
-      <c r="Y215" s="6" t="n"/>
+      <c r="X215" s="6" t="n"/>
     </row>
     <row r="216">
-      <c r="Y216" s="6" t="n"/>
+      <c r="X216" s="6" t="n"/>
     </row>
     <row r="217">
-      <c r="Y217" s="6" t="n"/>
+      <c r="X217" s="6" t="n"/>
     </row>
     <row r="218">
-      <c r="Y218" s="6" t="n"/>
+      <c r="X218" s="6" t="n"/>
     </row>
     <row r="219">
-      <c r="Y219" s="6" t="n"/>
+      <c r="X219" s="6" t="n"/>
     </row>
     <row r="220">
-      <c r="Y220" s="6" t="n"/>
+      <c r="X220" s="6" t="n"/>
     </row>
     <row r="221">
-      <c r="Y221" s="6" t="n"/>
+      <c r="X221" s="6" t="n"/>
     </row>
     <row r="222">
-      <c r="Y222" s="6" t="n"/>
+      <c r="X222" s="6" t="n"/>
     </row>
     <row r="223">
-      <c r="Y223" s="6" t="n"/>
+      <c r="X223" s="6" t="n"/>
     </row>
     <row r="224">
-      <c r="Y224" s="6" t="n"/>
+      <c r="X224" s="6" t="n"/>
     </row>
     <row r="225">
-      <c r="Y225" s="6" t="n"/>
+      <c r="X225" s="6" t="n"/>
     </row>
     <row r="226">
-      <c r="Y226" s="6" t="n"/>
+      <c r="X226" s="6" t="n"/>
     </row>
     <row r="227">
-      <c r="Y227" s="6" t="n"/>
+      <c r="X227" s="6" t="n"/>
     </row>
     <row r="228">
-      <c r="Y228" s="6" t="n"/>
+      <c r="X228" s="6" t="n"/>
     </row>
     <row r="229">
-      <c r="Y229" s="6" t="n"/>
+      <c r="X229" s="6" t="n"/>
     </row>
     <row r="230">
-      <c r="Y230" s="6" t="n"/>
+      <c r="X230" s="6" t="n"/>
     </row>
     <row r="231">
-      <c r="Y231" s="6" t="n"/>
+      <c r="X231" s="6" t="n"/>
     </row>
     <row r="232">
-      <c r="Y232" s="6" t="n"/>
+      <c r="X232" s="6" t="n"/>
     </row>
     <row r="233">
-      <c r="Y233" s="6" t="n"/>
+      <c r="X233" s="6" t="n"/>
     </row>
     <row r="234">
-      <c r="Y234" s="6" t="n"/>
+      <c r="X234" s="6" t="n"/>
     </row>
     <row r="235">
-      <c r="Y235" s="6" t="n"/>
+      <c r="X235" s="6" t="n"/>
     </row>
     <row r="236">
-      <c r="Y236" s="6" t="n"/>
+      <c r="X236" s="6" t="n"/>
     </row>
     <row r="237">
-      <c r="Y237" s="6" t="n"/>
+      <c r="X237" s="6" t="n"/>
     </row>
     <row r="238">
-      <c r="Y238" s="6" t="n"/>
+      <c r="X238" s="6" t="n"/>
     </row>
     <row r="239">
-      <c r="Y239" s="6" t="n"/>
+      <c r="X239" s="6" t="n"/>
     </row>
     <row r="240">
-      <c r="Y240" s="6" t="n"/>
+      <c r="X240" s="6" t="n"/>
     </row>
     <row r="241">
-      <c r="Y241" s="6" t="n"/>
+      <c r="X241" s="6" t="n"/>
     </row>
     <row r="242">
-      <c r="Y242" s="6" t="n"/>
+      <c r="X242" s="6" t="n"/>
     </row>
     <row r="243">
-      <c r="Y243" s="6" t="n"/>
+      <c r="X243" s="6" t="n"/>
     </row>
     <row r="244">
-      <c r="Y244" s="6" t="n"/>
+      <c r="X244" s="6" t="n"/>
     </row>
     <row r="245">
-      <c r="Y245" s="6" t="n"/>
+      <c r="X245" s="6" t="n"/>
     </row>
     <row r="246">
-      <c r="Y246" s="6" t="n"/>
+      <c r="X246" s="6" t="n"/>
     </row>
     <row r="247">
-      <c r="Y247" s="6" t="n"/>
+      <c r="X247" s="6" t="n"/>
     </row>
     <row r="248">
-      <c r="Y248" s="6" t="n"/>
+      <c r="X248" s="6" t="n"/>
     </row>
     <row r="249">
-      <c r="Y249" s="6" t="n"/>
+      <c r="X249" s="6" t="n"/>
     </row>
     <row r="250">
-      <c r="Y250" s="6" t="n"/>
+      <c r="X250" s="6" t="n"/>
     </row>
     <row r="251">
-      <c r="Y251" s="6" t="n"/>
+      <c r="X251" s="6" t="n"/>
     </row>
     <row r="252">
-      <c r="Y252" s="6" t="n"/>
+      <c r="X252" s="6" t="n"/>
     </row>
     <row r="253">
-      <c r="Y253" s="6" t="n"/>
+      <c r="X253" s="6" t="n"/>
     </row>
     <row r="254">
-      <c r="Y254" s="6" t="n"/>
+      <c r="X254" s="6" t="n"/>
     </row>
     <row r="255">
-      <c r="Y255" s="6" t="n"/>
+      <c r="X255" s="6" t="n"/>
     </row>
     <row r="256">
-      <c r="Y256" s="6" t="n"/>
+      <c r="X256" s="6" t="n"/>
     </row>
     <row r="257">
-      <c r="Y257" s="6" t="n"/>
+      <c r="X257" s="6" t="n"/>
     </row>
     <row r="258">
-      <c r="Y258" s="6" t="n"/>
+      <c r="X258" s="6" t="n"/>
     </row>
     <row r="259">
-      <c r="Y259" s="6" t="n"/>
+      <c r="X259" s="6" t="n"/>
     </row>
     <row r="260">
-      <c r="Y260" s="6" t="n"/>
+      <c r="X260" s="6" t="n"/>
     </row>
     <row r="261">
-      <c r="Y261" s="6" t="n"/>
+      <c r="X261" s="6" t="n"/>
     </row>
     <row r="262">
-      <c r="Y262" s="6" t="n"/>
+      <c r="X262" s="6" t="n"/>
     </row>
     <row r="263">
-      <c r="Y263" s="6" t="n"/>
+      <c r="X263" s="6" t="n"/>
     </row>
     <row r="264">
-      <c r="Y264" s="6" t="n"/>
+      <c r="X264" s="6" t="n"/>
     </row>
     <row r="265">
-      <c r="Y265" s="6" t="n"/>
+      <c r="X265" s="6" t="n"/>
     </row>
     <row r="266">
-      <c r="Y266" s="6" t="n"/>
+      <c r="X266" s="6" t="n"/>
     </row>
     <row r="267">
-      <c r="Y267" s="6" t="n"/>
+      <c r="X267" s="6" t="n"/>
     </row>
     <row r="268">
-      <c r="Y268" s="6" t="n"/>
+      <c r="X268" s="6" t="n"/>
     </row>
     <row r="269">
-      <c r="Y269" s="6" t="n"/>
+      <c r="X269" s="6" t="n"/>
     </row>
     <row r="270">
-      <c r="Y270" s="6" t="n"/>
+      <c r="X270" s="6" t="n"/>
     </row>
     <row r="271">
-      <c r="Y271" s="6" t="n"/>
+      <c r="X271" s="6" t="n"/>
     </row>
     <row r="272">
-      <c r="Y272" s="6" t="n"/>
+      <c r="X272" s="6" t="n"/>
     </row>
     <row r="273">
-      <c r="Y273" s="6" t="n"/>
+      <c r="X273" s="6" t="n"/>
     </row>
     <row r="274">
-      <c r="Y274" s="6" t="n"/>
+      <c r="X274" s="6" t="n"/>
     </row>
     <row r="275">
-      <c r="Y275" s="6" t="n"/>
+      <c r="X275" s="6" t="n"/>
     </row>
     <row r="276">
-      <c r="Y276" s="6" t="n"/>
+      <c r="X276" s="6" t="n"/>
     </row>
     <row r="277">
-      <c r="Y277" s="6" t="n"/>
+      <c r="X277" s="6" t="n"/>
     </row>
     <row r="278">
-      <c r="Y278" s="6" t="n"/>
+      <c r="X278" s="6" t="n"/>
     </row>
     <row r="279">
-      <c r="Y279" s="6" t="n"/>
+      <c r="X279" s="6" t="n"/>
     </row>
     <row r="280">
-      <c r="Y280" s="6" t="n"/>
+      <c r="X280" s="6" t="n"/>
     </row>
     <row r="281">
-      <c r="Y281" s="6" t="n"/>
+      <c r="X281" s="6" t="n"/>
     </row>
     <row r="282">
-      <c r="Y282" s="6" t="n"/>
+      <c r="X282" s="6" t="n"/>
     </row>
     <row r="283">
-      <c r="Y283" s="6" t="n"/>
+      <c r="X283" s="6" t="n"/>
     </row>
     <row r="284">
-      <c r="Y284" s="6" t="n"/>
+      <c r="X284" s="6" t="n"/>
     </row>
     <row r="285">
-      <c r="Y285" s="6" t="n"/>
+      <c r="X285" s="6" t="n"/>
     </row>
     <row r="286">
-      <c r="Y286" s="6" t="n"/>
+      <c r="X286" s="6" t="n"/>
     </row>
     <row r="287">
-      <c r="Y287" s="6" t="n"/>
+      <c r="X287" s="6" t="n"/>
     </row>
     <row r="288">
-      <c r="Y288" s="6" t="n"/>
+      <c r="X288" s="6" t="n"/>
     </row>
     <row r="289">
-      <c r="Y289" s="6" t="n"/>
+      <c r="X289" s="6" t="n"/>
     </row>
     <row r="290">
-      <c r="Y290" s="6" t="n"/>
+      <c r="X290" s="6" t="n"/>
     </row>
     <row r="291">
-      <c r="Y291" s="6" t="n"/>
+      <c r="X291" s="6" t="n"/>
     </row>
     <row r="292">
-      <c r="Y292" s="6" t="n"/>
+      <c r="X292" s="6" t="n"/>
     </row>
     <row r="293">
-      <c r="Y293" s="6" t="n"/>
+      <c r="X293" s="6" t="n"/>
     </row>
     <row r="294">
-      <c r="Y294" s="6" t="n"/>
+      <c r="X294" s="6" t="n"/>
     </row>
     <row r="295">
-      <c r="Y295" s="6" t="n"/>
+      <c r="X295" s="6" t="n"/>
     </row>
     <row r="296">
-      <c r="Y296" s="6" t="n"/>
+      <c r="X296" s="6" t="n"/>
     </row>
     <row r="297">
-      <c r="Y297" s="6" t="n"/>
+      <c r="X297" s="6" t="n"/>
     </row>
     <row r="298">
-      <c r="Y298" s="6" t="n"/>
+      <c r="X298" s="6" t="n"/>
     </row>
     <row r="299">
-      <c r="Y299" s="6" t="n"/>
+      <c r="X299" s="6" t="n"/>
     </row>
     <row r="300">
-      <c r="Y300" s="6" t="n"/>
+      <c r="X300" s="6" t="n"/>
     </row>
     <row r="301">
-      <c r="Y301" s="6" t="n"/>
+      <c r="X301" s="6" t="n"/>
     </row>
     <row r="302">
-      <c r="Y302" s="6" t="n"/>
+      <c r="X302" s="6" t="n"/>
     </row>
     <row r="303">
-      <c r="Y303" s="6" t="n"/>
+      <c r="X303" s="6" t="n"/>
     </row>
     <row r="304">
-      <c r="Y304" s="6" t="n"/>
+      <c r="X304" s="6" t="n"/>
     </row>
     <row r="305">
-      <c r="Y305" s="6" t="n"/>
+      <c r="X305" s="6" t="n"/>
     </row>
     <row r="306">
-      <c r="Y306" s="6" t="n"/>
+      <c r="X306" s="6" t="n"/>
     </row>
     <row r="307">
-      <c r="Y307" s="6" t="n"/>
+      <c r="X307" s="6" t="n"/>
     </row>
     <row r="308">
-      <c r="Y308" s="6" t="n"/>
+      <c r="X308" s="6" t="n"/>
     </row>
     <row r="309">
-      <c r="Y309" s="6" t="n"/>
+      <c r="X309" s="6" t="n"/>
     </row>
     <row r="310">
-      <c r="Y310" s="6" t="n"/>
+      <c r="X310" s="6" t="n"/>
     </row>
     <row r="311">
-      <c r="Y311" s="6" t="n"/>
+      <c r="X311" s="6" t="n"/>
     </row>
     <row r="312">
-      <c r="Y312" s="6" t="n"/>
+      <c r="X312" s="6" t="n"/>
     </row>
     <row r="313">
-      <c r="Y313" s="6" t="n"/>
+      <c r="X313" s="6" t="n"/>
     </row>
     <row r="314">
-      <c r="Y314" s="6" t="n"/>
+      <c r="X314" s="6" t="n"/>
     </row>
     <row r="315">
-      <c r="Y315" s="6" t="n"/>
+      <c r="X315" s="6" t="n"/>
     </row>
     <row r="316">
-      <c r="Y316" s="6" t="n"/>
+      <c r="X316" s="6" t="n"/>
     </row>
     <row r="317">
-      <c r="Y317" s="6" t="n"/>
+      <c r="X317" s="6" t="n"/>
     </row>
     <row r="318">
-      <c r="Y318" s="6" t="n"/>
+      <c r="X318" s="6" t="n"/>
     </row>
     <row r="319">
-      <c r="Y319" s="6" t="n"/>
+      <c r="X319" s="6" t="n"/>
     </row>
     <row r="320">
-      <c r="Y320" s="6" t="n"/>
+      <c r="X320" s="6" t="n"/>
     </row>
     <row r="321">
-      <c r="Y321" s="6" t="n"/>
+      <c r="X321" s="6" t="n"/>
     </row>
     <row r="322">
-      <c r="Y322" s="6" t="n"/>
+      <c r="X322" s="6" t="n"/>
     </row>
     <row r="323">
-      <c r="Y323" s="6" t="n"/>
+      <c r="X323" s="6" t="n"/>
     </row>
     <row r="324">
-      <c r="Y324" s="6" t="n"/>
+      <c r="X324" s="6" t="n"/>
     </row>
     <row r="325">
-      <c r="Y325" s="6" t="n"/>
+      <c r="X325" s="6" t="n"/>
     </row>
     <row r="326">
-      <c r="Y326" s="6" t="n"/>
+      <c r="X326" s="6" t="n"/>
     </row>
     <row r="327">
-      <c r="Y327" s="6" t="n"/>
+      <c r="X327" s="6" t="n"/>
     </row>
     <row r="328">
-      <c r="Y328" s="6" t="n"/>
+      <c r="X328" s="6" t="n"/>
     </row>
     <row r="329">
-      <c r="Y329" s="6" t="n"/>
+      <c r="X329" s="6" t="n"/>
     </row>
     <row r="330">
-      <c r="Y330" s="6" t="n"/>
+      <c r="X330" s="6" t="n"/>
     </row>
     <row r="331">
-      <c r="Y331" s="6" t="n"/>
+      <c r="X331" s="6" t="n"/>
     </row>
     <row r="332">
-      <c r="Y332" s="6" t="n"/>
+      <c r="X332" s="6" t="n"/>
     </row>
     <row r="333">
-      <c r="Y333" s="6" t="n"/>
+      <c r="X333" s="6" t="n"/>
     </row>
     <row r="334">
-      <c r="Y334" s="6" t="n"/>
+      <c r="X334" s="6" t="n"/>
     </row>
     <row r="335">
-      <c r="Y335" s="6" t="n"/>
+      <c r="X335" s="6" t="n"/>
     </row>
     <row r="336">
-      <c r="Y336" s="6" t="n"/>
+      <c r="X336" s="6" t="n"/>
     </row>
     <row r="337">
-      <c r="Y337" s="6" t="n"/>
+      <c r="X337" s="6" t="n"/>
     </row>
     <row r="338">
-      <c r="Y338" s="6" t="n"/>
+      <c r="X338" s="6" t="n"/>
     </row>
     <row r="339">
-      <c r="Y339" s="6" t="n"/>
+      <c r="X339" s="6" t="n"/>
     </row>
     <row r="340">
-      <c r="Y340" s="6" t="n"/>
+      <c r="X340" s="6" t="n"/>
     </row>
     <row r="341">
-      <c r="Y341" s="6" t="n"/>
+      <c r="X341" s="6" t="n"/>
     </row>
     <row r="342">
-      <c r="Y342" s="6" t="n"/>
+      <c r="X342" s="6" t="n"/>
     </row>
     <row r="343">
-      <c r="Y343" s="6" t="n"/>
+      <c r="X343" s="6" t="n"/>
     </row>
     <row r="344">
-      <c r="Y344" s="6" t="n"/>
+      <c r="X344" s="6" t="n"/>
     </row>
     <row r="345">
-      <c r="Y345" s="6" t="n"/>
+      <c r="X345" s="6" t="n"/>
     </row>
     <row r="346">
-      <c r="Y346" s="6" t="n"/>
+      <c r="X346" s="6" t="n"/>
     </row>
     <row r="347">
-      <c r="Y347" s="6" t="n"/>
+      <c r="X347" s="6" t="n"/>
     </row>
     <row r="348">
-      <c r="Y348" s="6" t="n"/>
+      <c r="X348" s="6" t="n"/>
     </row>
     <row r="349">
-      <c r="Y349" s="6" t="n"/>
+      <c r="X349" s="6" t="n"/>
     </row>
     <row r="350">
-      <c r="Y350" s="6" t="n"/>
+      <c r="X350" s="6" t="n"/>
     </row>
     <row r="351">
-      <c r="Y351" s="6" t="n"/>
+      <c r="X351" s="6" t="n"/>
     </row>
     <row r="352">
-      <c r="Y352" s="6" t="n"/>
+      <c r="X352" s="6" t="n"/>
     </row>
     <row r="353">
-      <c r="Y353" s="6" t="n"/>
+      <c r="X353" s="6" t="n"/>
     </row>
     <row r="354">
-      <c r="Y354" s="6" t="n"/>
+      <c r="X354" s="6" t="n"/>
     </row>
     <row r="355">
-      <c r="Y355" s="6" t="n"/>
+      <c r="X355" s="6" t="n"/>
     </row>
     <row r="356">
-      <c r="Y356" s="6" t="n"/>
+      <c r="X356" s="6" t="n"/>
     </row>
     <row r="357">
-      <c r="Y357" s="6" t="n"/>
+      <c r="X357" s="6" t="n"/>
     </row>
     <row r="358">
-      <c r="Y358" s="6" t="n"/>
+      <c r="X358" s="6" t="n"/>
     </row>
     <row r="359">
-      <c r="Y359" s="6" t="n"/>
+      <c r="X359" s="6" t="n"/>
     </row>
     <row r="360">
-      <c r="Y360" s="6" t="n"/>
+      <c r="X360" s="6" t="n"/>
     </row>
     <row r="361">
-      <c r="Y361" s="6" t="n"/>
+      <c r="X361" s="6" t="n"/>
     </row>
     <row r="362">
-      <c r="Y362" s="6" t="n"/>
+      <c r="X362" s="6" t="n"/>
     </row>
     <row r="363">
-      <c r="Y363" s="6" t="n"/>
+      <c r="X363" s="6" t="n"/>
     </row>
     <row r="364">
-      <c r="Y364" s="6" t="n"/>
+      <c r="X364" s="6" t="n"/>
     </row>
     <row r="365">
-      <c r="Y365" s="6" t="n"/>
+      <c r="X365" s="6" t="n"/>
     </row>
     <row r="366">
-      <c r="Y366" s="6" t="n"/>
+      <c r="X366" s="6" t="n"/>
     </row>
     <row r="367">
-      <c r="Y367" s="6" t="n"/>
+      <c r="X367" s="6" t="n"/>
     </row>
     <row r="368">
-      <c r="Y368" s="6" t="n"/>
+      <c r="X368" s="6" t="n"/>
     </row>
     <row r="369">
-      <c r="Y369" s="6" t="n"/>
+      <c r="X369" s="6" t="n"/>
     </row>
     <row r="370">
-      <c r="Y370" s="6" t="n"/>
+      <c r="X370" s="6" t="n"/>
     </row>
     <row r="371">
-      <c r="Y371" s="6" t="n"/>
+      <c r="X371" s="6" t="n"/>
     </row>
     <row r="372">
-      <c r="Y372" s="6" t="n"/>
+      <c r="X372" s="6" t="n"/>
     </row>
     <row r="373">
-      <c r="Y373" s="6" t="n"/>
+      <c r="X373" s="6" t="n"/>
     </row>
     <row r="374">
-      <c r="Y374" s="6" t="n"/>
+      <c r="X374" s="6" t="n"/>
     </row>
     <row r="375">
-      <c r="Y375" s="6" t="n"/>
+      <c r="X375" s="6" t="n"/>
     </row>
     <row r="376">
-      <c r="Y376" s="6" t="n"/>
+      <c r="X376" s="6" t="n"/>
     </row>
     <row r="377">
-      <c r="Y377" s="6" t="n"/>
+      <c r="X377" s="6" t="n"/>
     </row>
     <row r="378">
-      <c r="Y378" s="6" t="n"/>
+      <c r="X378" s="6" t="n"/>
     </row>
     <row r="379">
-      <c r="Y379" s="6" t="n"/>
+      <c r="X379" s="6" t="n"/>
     </row>
     <row r="380">
-      <c r="Y380" s="6" t="n"/>
+      <c r="X380" s="6" t="n"/>
     </row>
     <row r="381">
-      <c r="Y381" s="6" t="n"/>
+      <c r="X381" s="6" t="n"/>
     </row>
     <row r="382">
-      <c r="Y382" s="6" t="n"/>
+      <c r="X382" s="6" t="n"/>
     </row>
     <row r="383">
-      <c r="Y383" s="6" t="n"/>
+      <c r="X383" s="6" t="n"/>
     </row>
     <row r="384">
-      <c r="Y384" s="6" t="n"/>
+      <c r="X384" s="6" t="n"/>
     </row>
     <row r="385">
-      <c r="Y385" s="6" t="n"/>
+      <c r="X385" s="6" t="n"/>
     </row>
     <row r="386">
-      <c r="Y386" s="6" t="n"/>
+      <c r="X386" s="6" t="n"/>
     </row>
     <row r="387">
-      <c r="Y387" s="6" t="n"/>
+      <c r="X387" s="6" t="n"/>
     </row>
     <row r="388">
-      <c r="Y388" s="6" t="n"/>
+      <c r="X388" s="6" t="n"/>
     </row>
     <row r="389">
-      <c r="Y389" s="6" t="n"/>
+      <c r="X389" s="6" t="n"/>
     </row>
     <row r="390">
-      <c r="Y390" s="6" t="n"/>
+      <c r="X390" s="6" t="n"/>
     </row>
     <row r="391">
-      <c r="Y391" s="6" t="n"/>
+      <c r="X391" s="6" t="n"/>
     </row>
     <row r="392">
-      <c r="Y392" s="6" t="n"/>
+      <c r="X392" s="6" t="n"/>
     </row>
     <row r="393">
-      <c r="Y393" s="6" t="n"/>
+      <c r="X393" s="6" t="n"/>
     </row>
     <row r="394">
-      <c r="Y394" s="6" t="n"/>
+      <c r="X394" s="6" t="n"/>
     </row>
     <row r="395">
-      <c r="Y395" s="6" t="n"/>
+      <c r="X395" s="6" t="n"/>
     </row>
     <row r="396">
-      <c r="Y396" s="6" t="n"/>
+      <c r="X396" s="6" t="n"/>
     </row>
     <row r="397">
-      <c r="Y397" s="6" t="n"/>
+      <c r="X397" s="6" t="n"/>
     </row>
     <row r="398">
-      <c r="Y398" s="6" t="n"/>
+      <c r="X398" s="6" t="n"/>
     </row>
     <row r="399">
-      <c r="Y399" s="6" t="n"/>
+      <c r="X399" s="6" t="n"/>
     </row>
     <row r="400">
-      <c r="Y400" s="6" t="n"/>
+      <c r="X400" s="6" t="n"/>
     </row>
     <row r="401">
-      <c r="Y401" s="6" t="n"/>
+      <c r="X401" s="6" t="n"/>
     </row>
     <row r="402">
-      <c r="Y402" s="6" t="n"/>
+      <c r="X402" s="6" t="n"/>
     </row>
     <row r="403">
-      <c r="Y403" s="6" t="n"/>
+      <c r="X403" s="6" t="n"/>
     </row>
     <row r="404">
-      <c r="Y404" s="6" t="n"/>
+      <c r="X404" s="6" t="n"/>
     </row>
     <row r="405">
-      <c r="Y405" s="6" t="n"/>
+      <c r="X405" s="6" t="n"/>
     </row>
     <row r="406">
-      <c r="Y406" s="6" t="n"/>
+      <c r="X406" s="6" t="n"/>
     </row>
     <row r="407">
-      <c r="Y407" s="6" t="n"/>
+      <c r="X407" s="6" t="n"/>
     </row>
     <row r="408">
-      <c r="Y408" s="6" t="n"/>
+      <c r="X408" s="6" t="n"/>
     </row>
     <row r="409">
-      <c r="Y409" s="6" t="n"/>
+      <c r="X409" s="6" t="n"/>
     </row>
     <row r="410">
-      <c r="Y410" s="6" t="n"/>
+      <c r="X410" s="6" t="n"/>
     </row>
     <row r="411">
-      <c r="Y411" s="6" t="n"/>
+      <c r="X411" s="6" t="n"/>
     </row>
     <row r="412">
-      <c r="Y412" s="6" t="n"/>
+      <c r="X412" s="6" t="n"/>
     </row>
     <row r="413">
-      <c r="Y413" s="6" t="n"/>
+      <c r="X413" s="6" t="n"/>
     </row>
     <row r="414">
-      <c r="Y414" s="6" t="n"/>
+      <c r="X414" s="6" t="n"/>
     </row>
     <row r="415">
-      <c r="Y415" s="6" t="n"/>
+      <c r="X415" s="6" t="n"/>
     </row>
     <row r="416">
-      <c r="Y416" s="6" t="n"/>
+      <c r="X416" s="6" t="n"/>
     </row>
     <row r="417">
-      <c r="Y417" s="6" t="n"/>
+      <c r="X417" s="6" t="n"/>
     </row>
     <row r="418">
-      <c r="Y418" s="6" t="n"/>
+      <c r="X418" s="6" t="n"/>
     </row>
     <row r="419">
-      <c r="Y419" s="6" t="n"/>
+      <c r="X419" s="6" t="n"/>
     </row>
     <row r="420">
-      <c r="Y420" s="6" t="n"/>
+      <c r="X420" s="6" t="n"/>
     </row>
     <row r="421">
-      <c r="Y421" s="6" t="n"/>
+      <c r="X421" s="6" t="n"/>
     </row>
     <row r="422">
-      <c r="Y422" s="6" t="n"/>
+      <c r="X422" s="6" t="n"/>
     </row>
     <row r="423">
-      <c r="Y423" s="6" t="n"/>
+      <c r="X423" s="6" t="n"/>
     </row>
     <row r="424">
-      <c r="Y424" s="6" t="n"/>
+      <c r="X424" s="6" t="n"/>
     </row>
     <row r="425">
-      <c r="Y425" s="6" t="n"/>
+      <c r="X425" s="6" t="n"/>
     </row>
     <row r="426">
-      <c r="Y426" s="6" t="n"/>
+      <c r="X426" s="6" t="n"/>
     </row>
     <row r="427">
-      <c r="Y427" s="6" t="n"/>
+      <c r="X427" s="6" t="n"/>
     </row>
     <row r="428">
-      <c r="Y428" s="6" t="n"/>
+      <c r="X428" s="6" t="n"/>
     </row>
     <row r="429">
-      <c r="Y429" s="6" t="n"/>
+      <c r="X429" s="6" t="n"/>
     </row>
     <row r="430">
-      <c r="Y430" s="6" t="n"/>
+      <c r="X430" s="6" t="n"/>
     </row>
     <row r="431">
-      <c r="Y431" s="6" t="n"/>
+      <c r="X431" s="6" t="n"/>
     </row>
     <row r="432">
-      <c r="Y432" s="6" t="n"/>
+      <c r="X432" s="6" t="n"/>
     </row>
     <row r="433">
-      <c r="Y433" s="6" t="n"/>
+      <c r="X433" s="6" t="n"/>
     </row>
     <row r="434">
-      <c r="Y434" s="6" t="n"/>
+      <c r="X434" s="6" t="n"/>
     </row>
     <row r="435">
-      <c r="Y435" s="6" t="n"/>
+      <c r="X435" s="6" t="n"/>
     </row>
     <row r="436">
-      <c r="Y436" s="6" t="n"/>
+      <c r="X436" s="6" t="n"/>
     </row>
     <row r="437">
-      <c r="Y437" s="6" t="n"/>
+      <c r="X437" s="6" t="n"/>
     </row>
     <row r="438">
-      <c r="Y438" s="6" t="n"/>
+      <c r="X438" s="6" t="n"/>
     </row>
     <row r="439">
-      <c r="Y439" s="6" t="n"/>
+      <c r="X439" s="6" t="n"/>
     </row>
     <row r="440">
-      <c r="Y440" s="6" t="n"/>
+      <c r="X440" s="6" t="n"/>
     </row>
     <row r="441">
-      <c r="Y441" s="6" t="n"/>
+      <c r="X441" s="6" t="n"/>
     </row>
     <row r="442">
-      <c r="Y442" s="6" t="n"/>
+      <c r="X442" s="6" t="n"/>
     </row>
     <row r="443">
-      <c r="Y443" s="6" t="n"/>
+      <c r="X443" s="6" t="n"/>
     </row>
     <row r="444">
-      <c r="Y444" s="6" t="n"/>
+      <c r="X444" s="6" t="n"/>
     </row>
     <row r="445">
-      <c r="Y445" s="6" t="n"/>
+      <c r="X445" s="6" t="n"/>
     </row>
     <row r="446">
-      <c r="Y446" s="6" t="n"/>
+      <c r="X446" s="6" t="n"/>
     </row>
     <row r="447">
-      <c r="Y447" s="6" t="n"/>
+      <c r="X447" s="6" t="n"/>
     </row>
     <row r="448">
-      <c r="Y448" s="6" t="n"/>
+      <c r="X448" s="6" t="n"/>
     </row>
     <row r="449">
-      <c r="Y449" s="6" t="n"/>
+      <c r="X449" s="6" t="n"/>
     </row>
     <row r="450">
-      <c r="Y450" s="6" t="n"/>
+      <c r="X450" s="6" t="n"/>
     </row>
     <row r="451">
-      <c r="Y451" s="6" t="n"/>
+      <c r="X451" s="6" t="n"/>
     </row>
     <row r="452">
-      <c r="Y452" s="6" t="n"/>
+      <c r="X452" s="6" t="n"/>
     </row>
     <row r="453">
-      <c r="Y453" s="6" t="n"/>
+      <c r="X453" s="6" t="n"/>
     </row>
     <row r="454">
-      <c r="Y454" s="6" t="n"/>
+      <c r="X454" s="6" t="n"/>
     </row>
     <row r="455">
-      <c r="Y455" s="6" t="n"/>
+      <c r="X455" s="6" t="n"/>
     </row>
     <row r="456">
-      <c r="Y456" s="6" t="n"/>
+      <c r="X456" s="6" t="n"/>
     </row>
     <row r="457">
-      <c r="Y457" s="6" t="n"/>
+      <c r="X457" s="6" t="n"/>
     </row>
     <row r="458">
-      <c r="Y458" s="6" t="n"/>
+      <c r="X458" s="6" t="n"/>
     </row>
     <row r="459">
-      <c r="Y459" s="6" t="n"/>
+      <c r="X459" s="6" t="n"/>
     </row>
     <row r="460">
-      <c r="Y460" s="6" t="n"/>
+      <c r="X460" s="6" t="n"/>
     </row>
     <row r="461">
-      <c r="Y461" s="6" t="n"/>
+      <c r="X461" s="6" t="n"/>
     </row>
     <row r="462">
-      <c r="Y462" s="6" t="n"/>
+      <c r="X462" s="6" t="n"/>
     </row>
     <row r="463">
-      <c r="Y463" s="6" t="n"/>
+      <c r="X463" s="6" t="n"/>
     </row>
     <row r="464">
-      <c r="Y464" s="6" t="n"/>
+      <c r="X464" s="6" t="n"/>
     </row>
     <row r="465">
-      <c r="Y465" s="6" t="n"/>
+      <c r="X465" s="6" t="n"/>
     </row>
     <row r="466">
-      <c r="Y466" s="6" t="n"/>
+      <c r="X466" s="6" t="n"/>
     </row>
     <row r="467">
-      <c r="Y467" s="6" t="n"/>
+      <c r="X467" s="6" t="n"/>
     </row>
     <row r="468">
-      <c r="Y468" s="6" t="n"/>
+      <c r="X468" s="6" t="n"/>
     </row>
     <row r="469">
-      <c r="Y469" s="6" t="n"/>
+      <c r="X469" s="6" t="n"/>
     </row>
     <row r="470">
-      <c r="Y470" s="6" t="n"/>
+      <c r="X470" s="6" t="n"/>
     </row>
     <row r="471">
-      <c r="Y471" s="6" t="n"/>
+      <c r="X471" s="6" t="n"/>
     </row>
     <row r="472">
-      <c r="Y472" s="6" t="n"/>
+      <c r="X472" s="6" t="n"/>
     </row>
     <row r="473">
-      <c r="Y473" s="6" t="n"/>
+      <c r="X473" s="6" t="n"/>
     </row>
     <row r="474">
-      <c r="Y474" s="6" t="n"/>
+      <c r="X474" s="6" t="n"/>
     </row>
     <row r="475">
-      <c r="Y475" s="6" t="n"/>
+      <c r="X475" s="6" t="n"/>
     </row>
     <row r="476">
-      <c r="Y476" s="6" t="n"/>
+      <c r="X476" s="6" t="n"/>
     </row>
     <row r="477">
-      <c r="Y477" s="6" t="n"/>
+      <c r="X477" s="6" t="n"/>
     </row>
     <row r="478">
-      <c r="Y478" s="6" t="n"/>
+      <c r="X478" s="6" t="n"/>
     </row>
     <row r="479">
-      <c r="Y479" s="6" t="n"/>
+      <c r="X479" s="6" t="n"/>
     </row>
     <row r="480">
-      <c r="Y480" s="6" t="n"/>
+      <c r="X480" s="6" t="n"/>
     </row>
     <row r="481">
-      <c r="Y481" s="6" t="n"/>
+      <c r="X481" s="6" t="n"/>
     </row>
     <row r="482">
-      <c r="Y482" s="6" t="n"/>
+      <c r="X482" s="6" t="n"/>
     </row>
     <row r="483">
-      <c r="Y483" s="6" t="n"/>
+      <c r="X483" s="6" t="n"/>
     </row>
     <row r="484">
-      <c r="Y484" s="6" t="n"/>
+      <c r="X484" s="6" t="n"/>
     </row>
     <row r="485">
-      <c r="Y485" s="6" t="n"/>
+      <c r="X485" s="6" t="n"/>
     </row>
     <row r="486">
-      <c r="Y486" s="6" t="n"/>
+      <c r="X486" s="6" t="n"/>
     </row>
     <row r="487">
-      <c r="Y487" s="6" t="n"/>
+      <c r="X487" s="6" t="n"/>
     </row>
     <row r="488">
-      <c r="Y488" s="6" t="n"/>
+      <c r="X488" s="6" t="n"/>
     </row>
     <row r="489">
-      <c r="Y489" s="6" t="n"/>
+      <c r="X489" s="6" t="n"/>
     </row>
     <row r="490">
-      <c r="Y490" s="6" t="n"/>
+      <c r="X490" s="6" t="n"/>
     </row>
     <row r="491">
-      <c r="Y491" s="6" t="n"/>
+      <c r="X491" s="6" t="n"/>
     </row>
     <row r="492">
-      <c r="Y492" s="6" t="n"/>
+      <c r="X492" s="6" t="n"/>
     </row>
     <row r="493">
-      <c r="Y493" s="6" t="n"/>
+      <c r="X493" s="6" t="n"/>
     </row>
     <row r="494">
-      <c r="Y494" s="6" t="n"/>
+      <c r="X494" s="6" t="n"/>
     </row>
     <row r="495">
-      <c r="Y495" s="6" t="n"/>
+      <c r="X495" s="6" t="n"/>
     </row>
     <row r="496">
-      <c r="Y496" s="6" t="n"/>
+      <c r="X496" s="6" t="n"/>
     </row>
     <row r="497">
-      <c r="Y497" s="6" t="n"/>
+      <c r="X497" s="6" t="n"/>
     </row>
     <row r="498">
-      <c r="Y498" s="6" t="n"/>
+      <c r="X498" s="6" t="n"/>
     </row>
     <row r="499">
-      <c r="Y499" s="6" t="n"/>
+      <c r="X499" s="6" t="n"/>
     </row>
     <row r="500">
-      <c r="Y500" s="6" t="n"/>
+      <c r="X500" s="6" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="N2:N2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"employee,worker,student,trainee,contractor,freelance"</formula1>
+      <formula1>"hr.contract_type_employee,hr.contract_type_company_executive,hr.contract_type_interim,hr.contract_type_seasonal,hr.contract_type_apprenticeship,hr.contract_type_intern,hr.contract_type_student,hr.contract_type_thesis"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"male,female,other"</formula1>
+    <dataValidation sqref="R2:R2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"male,female"</formula1>
     </dataValidation>
-    <dataValidation sqref="AE2:AE2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AD2:AD2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"single,married,cohabitant,widower,divorced"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2727,7 +2716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3182,7 +3171,7 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>employee_type</t>
+          <t>employee_type_id/id</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -3197,17 +3186,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Selezione</t>
+          <t>ID esterno</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>employee</t>
+          <t>hr.contract_type_employee</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Default: employee.</t>
+          <t>Odoo 20: anagrafica hr.employee.type. Vedi foglio Valori.</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3260,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Odoo 19: data di efficacia della "versione" del dipendente. Vuoto = oggi.</t>
+          <t>Odoo 20: data di efficacia della "versione" del dipendente. Vuoto = oggi.</t>
         </is>
       </c>
     </row>
@@ -3310,12 +3299,12 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>ssnid</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>N. previdenziale</t>
+          <t>Sesso (legale)</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -3325,25 +3314,29 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Testo</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr"/>
+          <t>Selezione</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>male / female</t>
+        </is>
+      </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Matricola INPS / altro, se usato.</t>
+          <t>Sesso legale anagrafico (Odoo 20 ammette solo male/female).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>birthday</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Sesso</t>
+          <t>Data di nascita</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -3353,29 +3346,25 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Selezione</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>male / female / other</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>In Odoo 18 il campo si chiama gender.</t>
-        </is>
-      </c>
+          <t>1980-01-01</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>birthday</t>
+          <t>place_of_birth</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Data di nascita</t>
+          <t>Luogo di nascita</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -3385,12 +3374,12 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Testo</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>1980-01-01</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr"/>
@@ -3398,12 +3387,12 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>place_of_birth</t>
+          <t>country_of_birth/id</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Luogo di nascita</t>
+          <t>Paese di nascita</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -3413,12 +3402,12 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>ID esterno</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>base.it</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr"/>
@@ -3426,12 +3415,12 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>country_of_birth/id</t>
+          <t>country_id/id</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Paese di nascita</t>
+          <t>Nazionalità</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -3454,12 +3443,12 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>country_id/id</t>
+          <t>private_street</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Nazionalità</t>
+          <t>Indirizzo privato</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3469,25 +3458,21 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>ID esterno</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>base.it</t>
-        </is>
-      </c>
+          <t>Testo</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr"/>
       <c r="F28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>private_street</t>
+          <t>private_zip</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Indirizzo privato</t>
+          <t>CAP privato</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -3506,12 +3491,12 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>private_zip</t>
+          <t>private_city</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>CAP privato</t>
+          <t>Città privata</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -3530,12 +3515,12 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>private_city</t>
+          <t>private_state_id/id</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Città privata</t>
+          <t>Provincia privata</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -3545,21 +3530,29 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Testo</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr"/>
-      <c r="F31" s="9" t="inlineStr"/>
+          <t>ID esterno</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>base.state_it_rm</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Usare base.state_it_ + sigla provincia minuscola: base.state_it_mi (Milano), base.state_it_rm (Roma), base.state_it_to (Torino)...</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>private_state_id/id</t>
+          <t>private_country_id/id</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Provincia privata</t>
+          <t>Paese privato</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -3574,24 +3567,20 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>base.state_it_rm</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>Usare base.state_it_ + sigla provincia minuscola: base.state_it_mi (Milano), base.state_it_rm (Roma), base.state_it_to (Torino)...</t>
-        </is>
-      </c>
+          <t>base.it</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>private_country_id/id</t>
+          <t>private_email</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Paese privato</t>
+          <t>Email privata</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -3601,25 +3590,21 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>ID esterno</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>base.it</t>
-        </is>
-      </c>
+          <t>Testo</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr"/>
       <c r="F33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>private_email</t>
+          <t>private_phone</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Email privata</t>
+          <t>Telefono privato</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -3638,12 +3623,12 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>private_phone</t>
+          <t>marital</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Telefono privato</t>
+          <t>Stato civile</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
@@ -3653,21 +3638,29 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Testo</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr"/>
-      <c r="F35" s="9" t="inlineStr"/>
+          <t>Selezione</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Default single.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>marital</t>
+          <t>children</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Stato civile</t>
+          <t>Figli a carico</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
@@ -3677,29 +3670,25 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Selezione</t>
+          <t>Intero</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>single</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Default single.</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>children</t>
+          <t>emergency_contact</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Figli a carico</t>
+          <t>Contatto emergenza</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -3709,25 +3698,21 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Intero</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>Testo</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr"/>
       <c r="F37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>emergency_contact</t>
+          <t>emergency_phone</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Contatto emergenza</t>
+          <t>Tel. emergenza</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -3746,12 +3731,12 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>emergency_phone</t>
+          <t>category_ids</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Tel. emergenza</t>
+          <t>Etichette</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -3761,7 +3746,7 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Nomi separati da virgola</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr"/>
@@ -3770,12 +3755,12 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>category_ids</t>
+          <t>barcode</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Etichette</t>
+          <t>Badge ID</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
@@ -3785,37 +3770,139 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Nomi separati da virgola</t>
+          <t>Testo</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr"/>
-      <c r="F40" s="9" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>barcode</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>Badge ID</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>Facoltativo</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Testo</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr"/>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>Univoco.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>employee_type_id/id</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>hr.contract_type_employee</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dipendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>hr.contract_type_company_executive</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dirigente / amministratore</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>hr.contract_type_interim</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Interinale</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>hr.contract_type_seasonal</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Occasionale / stagionale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>hr.contract_type_apprenticeship</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Apprendista</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hr.contract_type_intern</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Stagista / tirocinante</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>hr.contract_type_student</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Studente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hr.contract_type_thesis</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tesista</t>
         </is>
       </c>
     </row>

</xml_diff>